<commit_message>
Dias de comienzo y final de las campayas
</commit_message>
<xml_diff>
--- a/Modelo_de_datos/Modelo.xlsx
+++ b/Modelo_de_datos/Modelo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\felix\Desktop\Bancosol\Modelo_de_datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD75843A-D20B-4371-A8C6-98FB959CBC69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{682FCA23-B2BD-4560-AB45-E3D6D85F5867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="56">
   <si>
     <t>ROL</t>
   </si>
@@ -181,6 +181,18 @@
   </si>
   <si>
     <t>PK,FK</t>
+  </si>
+  <si>
+    <t>Dia_comienzo</t>
+  </si>
+  <si>
+    <t>Dia_final</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>(Campañas no se puede superponer)</t>
   </si>
 </sst>
 </file>
@@ -292,7 +304,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -300,7 +312,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -659,10 +670,10 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
-      <c r="B7" s="7" t="s">
+      <c r="B7" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" t="s">
         <v>12</v>
       </c>
       <c r="D7" t="s">
@@ -706,13 +717,13 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="2"/>
-      <c r="B10" s="7" t="s">
+      <c r="B10" t="s">
         <v>3</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" t="s">
         <v>19</v>
       </c>
     </row>
@@ -750,28 +761,28 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
-      <c r="B13" s="7" t="s">
+      <c r="B13" t="s">
         <v>3</v>
       </c>
-      <c r="C13" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F13" s="7" t="s">
+      <c r="C13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" t="s">
         <v>14</v>
       </c>
-      <c r="G13" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="H13" s="7" t="s">
+      <c r="G13" t="s">
+        <v>12</v>
+      </c>
+      <c r="H13" t="s">
         <v>28</v>
       </c>
-      <c r="I13" s="7" t="s">
+      <c r="I13" t="s">
         <v>29</v>
       </c>
     </row>
@@ -799,6 +810,12 @@
       <c r="D18" t="s">
         <v>35</v>
       </c>
+      <c r="E18" t="s">
+        <v>52</v>
+      </c>
+      <c r="F18" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B19" t="s">
@@ -809,6 +826,15 @@
       </c>
       <c r="D19" t="s">
         <v>41</v>
+      </c>
+      <c r="E19" t="s">
+        <v>54</v>
+      </c>
+      <c r="F19" t="s">
+        <v>54</v>
+      </c>
+      <c r="G19" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Fix: Cambio del modelo de datos a unos atributos
</commit_message>
<xml_diff>
--- a/Modelo_de_datos/Modelo.xlsx
+++ b/Modelo_de_datos/Modelo.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\felix\Desktop\Bancosol\Modelo_de_datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{682FCA23-B2BD-4560-AB45-E3D6D85F5867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BC725CD-A163-49D1-8C3E-36C89947D689}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="65">
   <si>
     <t>ROL</t>
   </si>
@@ -193,6 +193,33 @@
   </si>
   <si>
     <t>(Campañas no se puede superponer)</t>
+  </si>
+  <si>
+    <t>ID_Capitan</t>
+  </si>
+  <si>
+    <t>FK(Usuario, rol capitan)</t>
+  </si>
+  <si>
+    <t>ID_destino</t>
+  </si>
+  <si>
+    <t>FK(usuario)</t>
+  </si>
+  <si>
+    <t>Fecha_creacion</t>
+  </si>
+  <si>
+    <t>timestamp</t>
+  </si>
+  <si>
+    <t>Mensaje</t>
+  </si>
+  <si>
+    <t>String(Not null)</t>
+  </si>
+  <si>
+    <t>FK(Usuario) rol coordinador</t>
   </si>
 </sst>
 </file>
@@ -304,7 +331,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -312,6 +339,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -598,13 +626,13 @@
     <col min="1" max="1" width="10.6640625" customWidth="1"/>
     <col min="2" max="2" width="12.5546875" customWidth="1"/>
     <col min="3" max="3" width="15.21875" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="12.109375" customWidth="1"/>
+    <col min="4" max="4" width="23.6640625" customWidth="1"/>
+    <col min="5" max="5" width="13.21875" customWidth="1"/>
     <col min="6" max="6" width="11.21875" customWidth="1"/>
     <col min="7" max="7" width="15.109375" customWidth="1"/>
     <col min="8" max="8" width="14.77734375" customWidth="1"/>
     <col min="9" max="9" width="24.44140625" customWidth="1"/>
-    <col min="10" max="10" width="12.33203125" customWidth="1"/>
+    <col min="10" max="10" width="20.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
@@ -758,6 +786,9 @@
       <c r="I12" s="4" t="s">
         <v>27</v>
       </c>
+      <c r="J12" s="7" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
@@ -785,6 +816,9 @@
       <c r="I13" t="s">
         <v>29</v>
       </c>
+      <c r="J13" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="14" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="3"/>
@@ -796,6 +830,29 @@
       <c r="B15" t="s">
         <v>1</v>
       </c>
+      <c r="C15" t="s">
+        <v>58</v>
+      </c>
+      <c r="D15" t="s">
+        <v>60</v>
+      </c>
+      <c r="E15" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B16" t="s">
+        <v>3</v>
+      </c>
+      <c r="C16" t="s">
+        <v>59</v>
+      </c>
+      <c r="D16" t="s">
+        <v>61</v>
+      </c>
+      <c r="E16" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
@@ -951,6 +1008,9 @@
       <c r="C27" t="s">
         <v>48</v>
       </c>
+      <c r="D27" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B28" t="s">
@@ -958,6 +1018,9 @@
       </c>
       <c r="C28" t="s">
         <v>51</v>
+      </c>
+      <c r="D28" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>